<commit_message>
feat: Implement lazy loading for game configuration and enhance Marble gameplay mechanics
Added a batch script for lazy loading JSON configurations into the project. Updated the ConfigSystem to load JSON data instead of byte buffers. Modified the Marble configuration XML to reflect new naming conventions and added JSON data files for Marble entities. Introduced new gameplay abilities and equipment classes to enhance the Marble gameplay experience.
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/marble.xlsx
+++ b/Configs/GameConfig/Datas/marble.xlsx
@@ -32,7 +32,7 @@
     <t>##var</t>
   </si>
   <si>
-    <t>id</t>
+    <t>config_id</t>
   </si>
   <si>
     <t>name</t>
@@ -276,30 +276,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="39">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF92D050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -653,7 +635,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -677,16 +659,16 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="10" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -695,89 +677,89 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -802,49 +784,43 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1">
@@ -1208,77 +1184,77 @@
       <c r="C2" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
-      <c r="J2" s="15"/>
-      <c r="K2" s="15"/>
-      <c r="L2" s="15"/>
-      <c r="M2" s="15"/>
-      <c r="N2" s="15"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
+      <c r="J2" s="14"/>
+      <c r="K2" s="14"/>
+      <c r="L2" s="14"/>
+      <c r="M2" s="14"/>
+      <c r="N2" s="14"/>
     </row>
     <row r="3" s="1" customFormat="1" spans="1:14">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="17"/>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18" t="s">
+      <c r="B3" s="15"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="19" t="s">
+      <c r="E3" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="19" t="s">
+      <c r="F3" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="G3" s="19" t="s">
+      <c r="G3" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="19" t="s">
+      <c r="H3" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="I3" s="19" t="s">
+      <c r="I3" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="J3" s="19" t="s">
+      <c r="J3" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="K3" s="19" t="s">
+      <c r="K3" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="L3" s="19" t="s">
+      <c r="L3" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="M3" s="19" t="s">
+      <c r="M3" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="N3" s="19" t="s">
+      <c r="N3" s="17" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="4" s="3" customFormat="1" spans="1:14">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="21"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
-      <c r="G4" s="23"/>
-      <c r="H4" s="23"/>
-      <c r="I4" s="23"/>
-      <c r="J4" s="23"/>
-      <c r="K4" s="23"/>
-      <c r="L4" s="23"/>
-      <c r="M4" s="23"/>
-      <c r="N4" s="23"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="21"/>
+      <c r="H4" s="21"/>
+      <c r="I4" s="21"/>
+      <c r="J4" s="21"/>
+      <c r="K4" s="21"/>
+      <c r="L4" s="21"/>
+      <c r="M4" s="21"/>
+      <c r="N4" s="21"/>
     </row>
     <row r="5" customHeight="1" spans="1:14">
       <c r="B5" s="5" t="s">

</xml_diff>

<commit_message>
feat: Add new equipment and marble configuration files for gameplay mechanics
Introduced new Excel and XML configuration files for equipment and marble entities, enhancing the game's ability to manage equipment attributes and marble properties. This update includes a new equipment definition schema and updates to the marble configuration to improve gameplay dynamics and flexibility.
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/marble.xlsx
+++ b/Configs/GameConfig/Datas/marble.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="25">
   <si>
     <t>##var</t>
   </si>
@@ -77,7 +77,7 @@
     <t>scale</t>
   </si>
   <si>
-    <t>lst_equipment_id</t>
+    <t>lst_equipment</t>
   </si>
   <si>
     <t>lst_ability_id</t>
@@ -86,7 +86,7 @@
     <t>##</t>
   </si>
   <si>
-    <t>Soldier</t>
+    <t>solider</t>
   </si>
   <si>
     <t>士兵</t>
@@ -95,7 +95,13 @@
     <t>0</t>
   </si>
   <si>
+    <t>sword,0,2</t>
+  </si>
+  <si>
     <t>1</t>
+  </si>
+  <si>
+    <t>sword,1,2</t>
   </si>
 </sst>
 </file>
@@ -759,7 +765,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -772,25 +778,19 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -811,7 +811,7 @@
     <xf numFmtId="49" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -823,7 +823,7 @@
     <xf numFmtId="49" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1142,182 +1142,188 @@
   <cols>
     <col min="1" max="1" width="9" style="4"/>
     <col min="2" max="2" width="9" style="5"/>
-    <col min="3" max="3" width="8.09090909090909" style="6" customWidth="1"/>
-    <col min="4" max="4" width="22.1818181818182" style="6" customWidth="1"/>
-    <col min="5" max="5" width="12.9090909090909" style="7" customWidth="1"/>
-    <col min="6" max="12" width="9" style="7"/>
-    <col min="13" max="13" width="18.5454545454545" style="7" customWidth="1"/>
-    <col min="14" max="14" width="16.2727272727273" style="7" customWidth="1"/>
+    <col min="3" max="3" width="8.09090909090909" style="4" customWidth="1"/>
+    <col min="4" max="4" width="22.1818181818182" style="4" customWidth="1"/>
+    <col min="5" max="5" width="12.9090909090909" style="6" customWidth="1"/>
+    <col min="6" max="12" width="9" style="6"/>
+    <col min="13" max="13" width="18.5454545454545" style="6" customWidth="1"/>
+    <col min="14" max="14" width="16.2727272727273" style="6" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:14">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
-      <c r="K1" s="11"/>
-      <c r="L1" s="11"/>
-      <c r="M1" s="11"/>
-      <c r="N1" s="11"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="9"/>
+      <c r="N1" s="9"/>
     </row>
     <row r="2" s="2" customFormat="1" spans="1:14">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="14" t="s">
+      <c r="D2" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="14"/>
-      <c r="L2" s="14"/>
-      <c r="M2" s="14"/>
-      <c r="N2" s="14"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+      <c r="M2" s="12"/>
+      <c r="N2" s="12"/>
     </row>
     <row r="3" s="1" customFormat="1" spans="1:14">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="15"/>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16" t="s">
+      <c r="B3" s="13"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="17" t="s">
+      <c r="E3" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="17" t="s">
+      <c r="F3" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="G3" s="17" t="s">
+      <c r="G3" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="17" t="s">
+      <c r="H3" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="I3" s="17" t="s">
+      <c r="I3" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="J3" s="17" t="s">
+      <c r="J3" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="K3" s="17" t="s">
+      <c r="K3" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="L3" s="17" t="s">
+      <c r="L3" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="M3" s="17" t="s">
+      <c r="M3" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="N3" s="17" t="s">
+      <c r="N3" s="15" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="4" s="3" customFormat="1" spans="1:14">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="21"/>
-      <c r="G4" s="21"/>
-      <c r="H4" s="21"/>
-      <c r="I4" s="21"/>
-      <c r="J4" s="21"/>
-      <c r="K4" s="21"/>
-      <c r="L4" s="21"/>
-      <c r="M4" s="21"/>
-      <c r="N4" s="21"/>
+      <c r="B4" s="17"/>
+      <c r="C4" s="18"/>
+      <c r="D4" s="18"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="19"/>
+      <c r="H4" s="19"/>
+      <c r="I4" s="19"/>
+      <c r="J4" s="19"/>
+      <c r="K4" s="19"/>
+      <c r="L4" s="19"/>
+      <c r="M4" s="19"/>
+      <c r="N4" s="19"/>
     </row>
     <row r="5" customHeight="1" spans="1:14">
       <c r="B5" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="6">
         <v>100</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5" s="6">
         <v>100</v>
       </c>
-      <c r="G5" s="7">
+      <c r="G5" s="6">
         <v>100</v>
       </c>
-      <c r="H5" s="7">
+      <c r="H5" s="6">
         <v>10</v>
       </c>
-      <c r="I5" s="7">
+      <c r="I5" s="6">
         <v>5</v>
       </c>
-      <c r="J5" s="7">
+      <c r="J5" s="6">
         <v>5</v>
       </c>
-      <c r="K5" s="7">
+      <c r="K5" s="6">
         <v>1</v>
       </c>
-      <c r="L5" s="7">
+      <c r="L5" s="6">
         <v>1</v>
+      </c>
+      <c r="M5" s="6" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:14">
-      <c r="D6" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="E6" s="7">
+      <c r="D6" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" s="6">
         <v>150</v>
       </c>
-      <c r="F6" s="7">
+      <c r="F6" s="6">
         <v>150</v>
       </c>
-      <c r="G6" s="7">
+      <c r="G6" s="6">
         <v>150</v>
       </c>
-      <c r="H6" s="7">
+      <c r="H6" s="6">
         <v>10</v>
       </c>
-      <c r="I6" s="7">
+      <c r="I6" s="6">
         <v>5</v>
       </c>
-      <c r="J6" s="7">
+      <c r="J6" s="6">
         <v>5</v>
       </c>
-      <c r="K6" s="7">
+      <c r="K6" s="6">
         <v>1</v>
       </c>
-      <c r="L6" s="7">
+      <c r="L6" s="6">
         <v>1</v>
+      </c>
+      <c r="M6" s="6" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Enhance Marble and Equipment configurations with new abilities and structural updates
Updated marble and equipment configuration files to introduce new abilities, including MarbleCloseToTargetAbility, and restructured existing configurations for improved gameplay dynamics. Adjusted XML and JSON files to reflect these changes, ensuring better integration with the combat system. Enhanced the ability system by categorizing abilities and refining the registration process, facilitating a more modular approach to gameplay mechanics.
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/marble.xlsx
+++ b/Configs/GameConfig/Datas/marble.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="27">
   <si>
     <t>##var</t>
   </si>
@@ -80,12 +80,15 @@
     <t>lst_equipment</t>
   </si>
   <si>
-    <t>lst_ability_id</t>
+    <t>lst_ability</t>
   </si>
   <si>
     <t>##</t>
   </si>
   <si>
+    <t>type,priority</t>
+  </si>
+  <si>
     <t>solider</t>
   </si>
   <si>
@@ -96,6 +99,9 @@
   </si>
   <si>
     <t>sword,0,2</t>
+  </si>
+  <si>
+    <t>close_to_target,0,3</t>
   </si>
   <si>
     <t>1</t>
@@ -494,7 +500,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -515,6 +521,39 @@
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -641,7 +680,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -653,34 +692,34 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -765,7 +804,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -792,19 +831,34 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -814,6 +868,12 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -824,6 +884,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1137,7 +1200,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="5"/>
   <cols>
     <col min="1" max="1" width="9" style="4"/>
@@ -1147,10 +1210,10 @@
     <col min="5" max="5" width="12.9090909090909" style="6" customWidth="1"/>
     <col min="6" max="12" width="9" style="6"/>
     <col min="13" max="13" width="18.5454545454545" style="6" customWidth="1"/>
-    <col min="14" max="14" width="16.2727272727273" style="6" customWidth="1"/>
+    <col min="14" max="14" width="51.5454545454545" style="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:14">
+    <row r="1" s="1" customFormat="1" spans="1:16">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -1163,108 +1226,114 @@
       <c r="D1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
-      <c r="K1" s="9"/>
-      <c r="L1" s="9"/>
-      <c r="M1" s="9"/>
-      <c r="N1" s="9"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
+      <c r="N1" s="10"/>
+      <c r="O1" s="11"/>
+      <c r="P1" s="11"/>
     </row>
-    <row r="2" s="2" customFormat="1" spans="1:14">
-      <c r="A2" s="10" t="s">
+    <row r="2" s="2" customFormat="1" spans="1:16">
+      <c r="A2" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
-      <c r="M2" s="12"/>
-      <c r="N2" s="12"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
+      <c r="J2" s="15"/>
+      <c r="K2" s="15"/>
+      <c r="L2" s="15"/>
+      <c r="M2" s="15"/>
+      <c r="N2" s="16"/>
     </row>
-    <row r="3" s="1" customFormat="1" spans="1:14">
-      <c r="A3" s="9" t="s">
+    <row r="3" s="1" customFormat="1" spans="1:16">
+      <c r="A3" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14" t="s">
+      <c r="B3" s="18"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="E3" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="G3" s="15" t="s">
+      <c r="G3" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="15" t="s">
+      <c r="H3" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="I3" s="15" t="s">
+      <c r="I3" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="J3" s="15" t="s">
+      <c r="J3" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="K3" s="15" t="s">
+      <c r="K3" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="L3" s="15" t="s">
+      <c r="L3" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="M3" s="15" t="s">
+      <c r="M3" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="N3" s="15" t="s">
+      <c r="N3" s="21" t="s">
         <v>17</v>
       </c>
+      <c r="O3" s="22"/>
+      <c r="P3" s="22"/>
     </row>
-    <row r="4" s="3" customFormat="1" spans="1:14">
-      <c r="A4" s="16" t="s">
+    <row r="4" s="3" customFormat="1" spans="1:16">
+      <c r="A4" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="17"/>
-      <c r="C4" s="18"/>
-      <c r="D4" s="18"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
-      <c r="G4" s="19"/>
-      <c r="H4" s="19"/>
-      <c r="I4" s="19"/>
-      <c r="J4" s="19"/>
-      <c r="K4" s="19"/>
-      <c r="L4" s="19"/>
-      <c r="M4" s="19"/>
-      <c r="N4" s="19"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="25"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="26"/>
+      <c r="H4" s="26"/>
+      <c r="I4" s="26"/>
+      <c r="J4" s="26"/>
+      <c r="K4" s="26"/>
+      <c r="L4" s="26"/>
+      <c r="M4" s="26"/>
+      <c r="N4" s="27" t="s">
+        <v>19</v>
+      </c>
     </row>
-    <row r="5" customHeight="1" spans="1:14">
+    <row r="5" customHeight="1" spans="1:16">
       <c r="B5" s="5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E5" s="6">
         <v>100</v>
@@ -1291,12 +1360,15 @@
         <v>1</v>
       </c>
       <c r="M5" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="N5" s="6" t="s">
+        <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:14">
+    <row r="6" spans="1:16">
       <c r="D6" s="4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E6" s="6">
         <v>150</v>
@@ -1323,6 +1395,9 @@
         <v>1</v>
       </c>
       <c r="M6" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N6" s="6" t="s">
         <v>24</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Add new shield equipment and marble configuration updates
Introduced a new shield prefab and associated metadata to enhance the equipment system. Updated the marble configuration to include new abilities and improved gameplay dynamics. Added a new Excel file for marble data and modified existing JSON configurations to support the integration of the shield and its abilities, ensuring better gameplay mechanics and modularity.
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/marble.xlsx
+++ b/Configs/GameConfig/Datas/marble.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="29">
   <si>
     <t>##var</t>
   </si>
@@ -101,6 +101,9 @@
     <t>sword,0,2</t>
   </si>
   <si>
+    <t>shield,0,1</t>
+  </si>
+  <si>
     <t>close_to_target,0,3</t>
   </si>
   <si>
@@ -108,6 +111,9 @@
   </si>
   <si>
     <t>sword,1,2</t>
+  </si>
+  <si>
+    <t>shield,1,1</t>
   </si>
 </sst>
 </file>
@@ -500,7 +506,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -528,6 +534,32 @@
         <color auto="1"/>
       </left>
       <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
       <top/>
       <bottom/>
       <diagonal/>
@@ -549,11 +581,31 @@
       <left style="thin">
         <color auto="1"/>
       </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="thin">
         <color auto="1"/>
       </right>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -680,7 +732,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -692,34 +744,34 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -804,7 +856,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -826,18 +878,27 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -850,10 +911,13 @@
     <xf numFmtId="49" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -868,7 +932,13 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -886,7 +956,10 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1200,7 +1273,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:P6"/>
+  <dimension ref="A1:Q6"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="5"/>
   <cols>
     <col min="1" max="1" width="9" style="4"/>
@@ -1208,124 +1281,129 @@
     <col min="3" max="3" width="8.09090909090909" style="4" customWidth="1"/>
     <col min="4" max="4" width="22.1818181818182" style="4" customWidth="1"/>
     <col min="5" max="5" width="12.9090909090909" style="6" customWidth="1"/>
-    <col min="6" max="12" width="9" style="6"/>
-    <col min="13" max="13" width="18.5454545454545" style="6" customWidth="1"/>
-    <col min="14" max="14" width="51.5454545454545" style="6" customWidth="1"/>
+    <col min="6" max="11" width="9" style="6"/>
+    <col min="12" max="12" width="9" style="7"/>
+    <col min="13" max="14" width="18.5454545454545" style="6" customWidth="1"/>
+    <col min="15" max="15" width="51.5454545454545" style="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:16">
-      <c r="A1" s="7" t="s">
+    <row r="1" s="1" customFormat="1" spans="1:17">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="10"/>
-      <c r="K1" s="10"/>
-      <c r="L1" s="10"/>
-      <c r="M1" s="10"/>
-      <c r="N1" s="10"/>
-      <c r="O1" s="11"/>
-      <c r="P1" s="11"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="13"/>
+      <c r="N1" s="13"/>
+      <c r="O1" s="12"/>
+      <c r="P1" s="14"/>
+      <c r="Q1" s="14"/>
     </row>
-    <row r="2" s="2" customFormat="1" spans="1:16">
-      <c r="A2" s="12" t="s">
+    <row r="2" s="2" customFormat="1" spans="1:17">
+      <c r="A2" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
-      <c r="J2" s="15"/>
-      <c r="K2" s="15"/>
-      <c r="L2" s="15"/>
-      <c r="M2" s="15"/>
-      <c r="N2" s="16"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
+      <c r="J2" s="18"/>
+      <c r="K2" s="18"/>
+      <c r="L2" s="19"/>
+      <c r="M2" s="17"/>
+      <c r="N2" s="17"/>
+      <c r="O2" s="20"/>
     </row>
-    <row r="3" s="1" customFormat="1" spans="1:16">
-      <c r="A3" s="17" t="s">
+    <row r="3" s="1" customFormat="1" spans="1:17">
+      <c r="A3" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="18"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19" t="s">
+      <c r="B3" s="22"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="20" t="s">
+      <c r="E3" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="20" t="s">
+      <c r="F3" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="G3" s="20" t="s">
+      <c r="G3" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="20" t="s">
+      <c r="H3" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="I3" s="20" t="s">
+      <c r="I3" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="J3" s="20" t="s">
+      <c r="J3" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="K3" s="20" t="s">
+      <c r="K3" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="L3" s="20" t="s">
+      <c r="L3" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="M3" s="20" t="s">
+      <c r="M3" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="N3" s="21" t="s">
+      <c r="N3" s="26"/>
+      <c r="O3" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="O3" s="22"/>
-      <c r="P3" s="22"/>
+      <c r="P3" s="28"/>
+      <c r="Q3" s="28"/>
     </row>
-    <row r="4" s="3" customFormat="1" spans="1:16">
-      <c r="A4" s="23" t="s">
+    <row r="4" s="3" customFormat="1" spans="1:17">
+      <c r="A4" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="24"/>
-      <c r="C4" s="25"/>
-      <c r="D4" s="25"/>
-      <c r="E4" s="26"/>
-      <c r="F4" s="26"/>
-      <c r="G4" s="26"/>
-      <c r="H4" s="26"/>
-      <c r="I4" s="26"/>
-      <c r="J4" s="26"/>
-      <c r="K4" s="26"/>
-      <c r="L4" s="26"/>
-      <c r="M4" s="26"/>
-      <c r="N4" s="27" t="s">
+      <c r="B4" s="30"/>
+      <c r="C4" s="31"/>
+      <c r="D4" s="31"/>
+      <c r="E4" s="32"/>
+      <c r="F4" s="32"/>
+      <c r="G4" s="32"/>
+      <c r="H4" s="32"/>
+      <c r="I4" s="32"/>
+      <c r="J4" s="32"/>
+      <c r="K4" s="32"/>
+      <c r="L4" s="33"/>
+      <c r="M4" s="32"/>
+      <c r="N4" s="32"/>
+      <c r="O4" s="34" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="5" customHeight="1" spans="1:16">
+    <row r="5" customHeight="1" spans="1:17">
       <c r="B5" s="5" t="s">
         <v>20</v>
       </c>
@@ -1356,7 +1434,7 @@
       <c r="K5" s="6">
         <v>1</v>
       </c>
-      <c r="L5" s="6">
+      <c r="L5" s="7">
         <v>1</v>
       </c>
       <c r="M5" s="6" t="s">
@@ -1365,10 +1443,13 @@
       <c r="N5" s="6" t="s">
         <v>24</v>
       </c>
+      <c r="O5" s="8" t="s">
+        <v>25</v>
+      </c>
     </row>
-    <row r="6" spans="1:16">
+    <row r="6" spans="1:17">
       <c r="D6" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E6" s="6">
         <v>150</v>
@@ -1391,20 +1472,24 @@
       <c r="K6" s="6">
         <v>1</v>
       </c>
-      <c r="L6" s="6">
+      <c r="L6" s="7">
         <v>1</v>
       </c>
       <c r="M6" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="N6" s="6" t="s">
-        <v>24</v>
+        <v>28</v>
+      </c>
+      <c r="O6" s="8" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="D1:N1"/>
-    <mergeCell ref="D2:N2"/>
+  <mergeCells count="3">
+    <mergeCell ref="D1:O1"/>
+    <mergeCell ref="D2:O2"/>
+    <mergeCell ref="M3:N3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
feat: Introduce new equipment configurations and enums for enhanced combat mechanics
Added new equipment configurations for swords and shields, including detailed level configurations and abilities. Introduced EnumEquipmentSlot and EnumCombineType enums to standardize equipment slot management and ability combination strategies. Updated XML and JSON files to reflect these changes, ensuring better integration with the combat system and improved gameplay dynamics.
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/marble.xlsx
+++ b/Configs/GameConfig/Datas/marble.xlsx
@@ -98,22 +98,22 @@
     <t>0</t>
   </si>
   <si>
-    <t>sword,0,2</t>
-  </si>
-  <si>
-    <t>shield,0,1</t>
-  </si>
-  <si>
-    <t>close_to_target,0,5</t>
+    <t>sword,0,right</t>
+  </si>
+  <si>
+    <t>shield,0,left</t>
+  </si>
+  <si>
+    <t>close_to_target,1000,combine,5</t>
   </si>
   <si>
     <t>1</t>
   </si>
   <si>
-    <t>sword,1,2</t>
-  </si>
-  <si>
-    <t>shield,1,1</t>
+    <t>sword,1,right</t>
+  </si>
+  <si>
+    <t>shield,1,left</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
feat: Enhance marble abilities with new configurations and physics adjustments
Added new ability configurations for MarbleCloseToTarget and MarbleDefaultRotate, including properties for target speed and acceleration. Updated XML and JSON files to reflect these changes, ensuring better integration with the combat system. Adjusted Rigidbody2D properties for marbles, swords, and shields to improve physics interactions, enhancing overall gameplay dynamics.
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/marble.xlsx
+++ b/Configs/GameConfig/Datas/marble.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="30">
   <si>
     <t>##var</t>
   </si>
@@ -104,7 +104,10 @@
     <t>shield,0,left</t>
   </si>
   <si>
-    <t>close_to_target,1000,combine,5</t>
+    <t>close_to_target,1000,combine,5,10,10</t>
+  </si>
+  <si>
+    <t>default_rotate, 1000, combine, 180, 180</t>
   </si>
   <si>
     <t>1</t>
@@ -506,7 +509,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="17">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -543,19 +546,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color auto="1"/>
       </left>
@@ -582,26 +572,6 @@
         <color auto="1"/>
       </left>
       <right/>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
       <top/>
       <bottom style="thin">
         <color auto="1"/>
@@ -732,7 +702,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -744,34 +714,34 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -856,7 +826,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -881,16 +851,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -911,15 +878,12 @@
     <xf numFmtId="49" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="2" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -938,7 +902,10 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -959,7 +926,7 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1273,7 +1240,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:Q6"/>
+  <dimension ref="A1:R6"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="5"/>
   <cols>
     <col min="1" max="1" width="9" style="4"/>
@@ -1284,126 +1251,131 @@
     <col min="6" max="11" width="9" style="6"/>
     <col min="12" max="12" width="9" style="7"/>
     <col min="13" max="14" width="18.5454545454545" style="6" customWidth="1"/>
-    <col min="15" max="15" width="51.5454545454545" style="8" customWidth="1"/>
+    <col min="15" max="15" width="42.2727272727273" style="6" customWidth="1"/>
+    <col min="16" max="16" width="51.5454545454545" style="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:17">
-      <c r="A1" s="9" t="s">
+    <row r="1" s="1" customFormat="1" spans="1:18">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="13"/>
-      <c r="N1" s="13"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
+      <c r="J1" s="11"/>
+      <c r="K1" s="11"/>
+      <c r="L1" s="11"/>
+      <c r="M1" s="12"/>
+      <c r="N1" s="12"/>
       <c r="O1" s="12"/>
-      <c r="P1" s="14"/>
-      <c r="Q1" s="14"/>
+      <c r="P1" s="12"/>
+      <c r="Q1" s="13"/>
+      <c r="R1" s="13"/>
     </row>
-    <row r="2" s="2" customFormat="1" spans="1:17">
-      <c r="A2" s="15" t="s">
+    <row r="2" s="2" customFormat="1" spans="1:18">
+      <c r="A2" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-      <c r="I2" s="18"/>
-      <c r="J2" s="18"/>
-      <c r="K2" s="18"/>
-      <c r="L2" s="19"/>
-      <c r="M2" s="17"/>
-      <c r="N2" s="17"/>
-      <c r="O2" s="20"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="17"/>
+      <c r="L2" s="18"/>
+      <c r="M2" s="16"/>
+      <c r="N2" s="16"/>
+      <c r="O2" s="16"/>
+      <c r="P2" s="16"/>
     </row>
-    <row r="3" s="1" customFormat="1" spans="1:17">
-      <c r="A3" s="21" t="s">
+    <row r="3" s="1" customFormat="1" spans="1:18">
+      <c r="A3" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="23"/>
-      <c r="D3" s="23" t="s">
+      <c r="B3" s="20"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="24" t="s">
+      <c r="E3" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="24" t="s">
+      <c r="F3" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="G3" s="24" t="s">
+      <c r="G3" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="24" t="s">
+      <c r="H3" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="I3" s="24" t="s">
+      <c r="I3" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="J3" s="24" t="s">
+      <c r="J3" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="K3" s="24" t="s">
+      <c r="K3" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="L3" s="25" t="s">
+      <c r="L3" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="M3" s="26" t="s">
+      <c r="M3" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="N3" s="26"/>
-      <c r="O3" s="27" t="s">
+      <c r="N3" s="24"/>
+      <c r="O3" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="P3" s="28"/>
-      <c r="Q3" s="28"/>
+      <c r="P3" s="26"/>
+      <c r="Q3" s="27"/>
+      <c r="R3" s="27"/>
     </row>
-    <row r="4" s="3" customFormat="1" spans="1:17">
-      <c r="A4" s="29" t="s">
+    <row r="4" s="3" customFormat="1" spans="1:18">
+      <c r="A4" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="30"/>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="32"/>
-      <c r="F4" s="32"/>
-      <c r="G4" s="32"/>
-      <c r="H4" s="32"/>
-      <c r="I4" s="32"/>
-      <c r="J4" s="32"/>
-      <c r="K4" s="32"/>
-      <c r="L4" s="33"/>
-      <c r="M4" s="32"/>
-      <c r="N4" s="32"/>
-      <c r="O4" s="34" t="s">
+      <c r="B4" s="29"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="31"/>
+      <c r="F4" s="31"/>
+      <c r="G4" s="31"/>
+      <c r="H4" s="31"/>
+      <c r="I4" s="31"/>
+      <c r="J4" s="31"/>
+      <c r="K4" s="31"/>
+      <c r="L4" s="32"/>
+      <c r="M4" s="31"/>
+      <c r="N4" s="31"/>
+      <c r="O4" s="31" t="s">
         <v>19</v>
       </c>
+      <c r="P4" s="33"/>
     </row>
-    <row r="5" customHeight="1" spans="1:17">
+    <row r="5" customHeight="1" spans="1:18">
       <c r="B5" s="5" t="s">
         <v>20</v>
       </c>
@@ -1443,13 +1415,16 @@
       <c r="N5" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="O5" s="8" t="s">
+      <c r="O5" s="6" t="s">
         <v>25</v>
       </c>
+      <c r="P5" s="6" t="s">
+        <v>26</v>
+      </c>
     </row>
-    <row r="6" spans="1:17">
+    <row r="6" spans="1:18">
       <c r="D6" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E6" s="6">
         <v>150</v>
@@ -1476,20 +1451,24 @@
         <v>1</v>
       </c>
       <c r="M6" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="N6" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="O6" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="O6" s="6" t="s">
         <v>25</v>
+      </c>
+      <c r="P6" s="6" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="D1:O1"/>
-    <mergeCell ref="D2:O2"/>
+  <mergeCells count="4">
+    <mergeCell ref="D1:P1"/>
+    <mergeCell ref="D2:P2"/>
     <mergeCell ref="M3:N3"/>
+    <mergeCell ref="O3:P3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
feat: Introduce MarbleDashAbility and timing configurations for enhanced gameplay
Added the MarbleDashAbility with properties for target speed, acceleration, and timing configurations, including FixedAbilityTimingConfig. Updated XML and JSON files to reflect these new abilities, ensuring better integration with the combat system. Enhanced the ability management system to support the new dash mechanics, improving overall gameplay dynamics.
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/marble.xlsx
+++ b/Configs/GameConfig/Datas/marble.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="31">
   <si>
     <t>##var</t>
   </si>
@@ -80,7 +80,7 @@
     <t>lst_equipment</t>
   </si>
   <si>
-    <t>lst_ability</t>
+    <t>lst_ability#format=lite</t>
   </si>
   <si>
     <t>##</t>
@@ -104,10 +104,13 @@
     <t>shield,0,left</t>
   </si>
   <si>
-    <t>close_to_target,1000,combine,5,10,10</t>
-  </si>
-  <si>
-    <t>default_rotate, 1000, combine, 180, 180</t>
+    <t>{close_to_target,1000,combine,5,10,10}</t>
+  </si>
+  <si>
+    <t>{default_rotate, 1000, combine, 180, 180}</t>
+  </si>
+  <si>
+    <t>{dash,2000,combine,20,20,false,{fixed_timing,1,3,true}}</t>
   </si>
   <si>
     <t>1</t>
@@ -902,13 +905,13 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -926,7 +929,7 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1240,8 +1243,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:R6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="5"/>
+  <dimension ref="A1:R7"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="6"/>
   <cols>
     <col min="1" max="1" width="9" style="4"/>
     <col min="2" max="2" width="9" style="5"/>
@@ -1251,8 +1254,10 @@
     <col min="6" max="11" width="9" style="6"/>
     <col min="12" max="12" width="9" style="7"/>
     <col min="13" max="14" width="18.5454545454545" style="6" customWidth="1"/>
-    <col min="15" max="15" width="42.2727272727273" style="6" customWidth="1"/>
-    <col min="16" max="16" width="51.5454545454545" style="6" customWidth="1"/>
+    <col min="15" max="15" width="168.636363636364" style="6" customWidth="1"/>
+    <col min="16" max="16" width="47.1818181818182" customWidth="1"/>
+    <col min="17" max="17" width="50.8181818181818" customWidth="1"/>
+    <col min="18" max="18" width="66.8181818181818" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:18">
@@ -1279,9 +1284,8 @@
       <c r="M1" s="12"/>
       <c r="N1" s="12"/>
       <c r="O1" s="12"/>
-      <c r="P1" s="12"/>
+      <c r="P1" s="13"/>
       <c r="Q1" s="13"/>
-      <c r="R1" s="13"/>
     </row>
     <row r="2" s="2" customFormat="1" spans="1:18">
       <c r="A2" s="14" t="s">
@@ -1307,7 +1311,6 @@
       <c r="M2" s="16"/>
       <c r="N2" s="16"/>
       <c r="O2" s="16"/>
-      <c r="P2" s="16"/>
     </row>
     <row r="3" s="1" customFormat="1" spans="1:18">
       <c r="A3" s="19" t="s">
@@ -1350,90 +1353,68 @@
         <v>17</v>
       </c>
       <c r="P3" s="26"/>
-      <c r="Q3" s="27"/>
-      <c r="R3" s="27"/>
+      <c r="Q3" s="26"/>
     </row>
-    <row r="4" s="3" customFormat="1" spans="1:18">
-      <c r="A4" s="28" t="s">
+    <row r="4" s="1" customFormat="1" spans="1:18">
+      <c r="A4" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="20"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
+      <c r="G4" s="22"/>
+      <c r="H4" s="22"/>
+      <c r="I4" s="22"/>
+      <c r="J4" s="22"/>
+      <c r="K4" s="22"/>
+      <c r="L4" s="23"/>
+      <c r="M4" s="24"/>
+      <c r="N4" s="24"/>
+      <c r="O4" s="27"/>
+      <c r="P4" s="26"/>
+      <c r="Q4" s="26"/>
+    </row>
+    <row r="5" s="3" customFormat="1" spans="1:18">
+      <c r="A5" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="29"/>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="31"/>
-      <c r="F4" s="31"/>
-      <c r="G4" s="31"/>
-      <c r="H4" s="31"/>
-      <c r="I4" s="31"/>
-      <c r="J4" s="31"/>
-      <c r="K4" s="31"/>
-      <c r="L4" s="32"/>
-      <c r="M4" s="31"/>
-      <c r="N4" s="31"/>
-      <c r="O4" s="31" t="s">
+      <c r="B5" s="29"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="31"/>
+      <c r="F5" s="31"/>
+      <c r="G5" s="31"/>
+      <c r="H5" s="31"/>
+      <c r="I5" s="31"/>
+      <c r="J5" s="31"/>
+      <c r="K5" s="31"/>
+      <c r="L5" s="32"/>
+      <c r="M5" s="31"/>
+      <c r="N5" s="31"/>
+      <c r="O5" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="P4" s="33"/>
     </row>
-    <row r="5" customHeight="1" spans="1:18">
-      <c r="B5" s="5" t="s">
+    <row r="6" customHeight="1" spans="1:18">
+      <c r="B6" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C6" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D6" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E6" s="6">
         <v>100</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F6" s="6">
         <v>100</v>
       </c>
-      <c r="G5" s="6">
+      <c r="G6" s="6">
         <v>100</v>
-      </c>
-      <c r="H5" s="6">
-        <v>10</v>
-      </c>
-      <c r="I5" s="6">
-        <v>5</v>
-      </c>
-      <c r="J5" s="6">
-        <v>8</v>
-      </c>
-      <c r="K5" s="6">
-        <v>1</v>
-      </c>
-      <c r="L5" s="7">
-        <v>1</v>
-      </c>
-      <c r="M5" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="N5" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="O5" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="P5" s="6" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18">
-      <c r="D6" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E6" s="6">
-        <v>150</v>
-      </c>
-      <c r="F6" s="6">
-        <v>150</v>
-      </c>
-      <c r="G6" s="6">
-        <v>150</v>
       </c>
       <c r="H6" s="6">
         <v>10</v>
@@ -1451,24 +1432,78 @@
         <v>1</v>
       </c>
       <c r="M6" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N6" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="O6" s="6" t="str">
+        <f>_xlfn.CONCAT("{",_xlfn.TEXTJOIN(",",TRUE,P6:R6),"}")</f>
+        <v>{{close_to_target,1000,combine,5,10,10},{default_rotate, 1000, combine, 180, 180},{dash,2000,combine,20,20,false,{fixed_timing,1,3,true}}}</v>
+      </c>
+      <c r="P6" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q6" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="R6" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18">
+      <c r="D7" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="N6" s="6" t="s">
+      <c r="E7" s="6">
+        <v>150</v>
+      </c>
+      <c r="F7" s="6">
+        <v>150</v>
+      </c>
+      <c r="G7" s="6">
+        <v>150</v>
+      </c>
+      <c r="H7" s="6">
+        <v>10</v>
+      </c>
+      <c r="I7" s="6">
+        <v>5</v>
+      </c>
+      <c r="J7" s="6">
+        <v>8</v>
+      </c>
+      <c r="K7" s="6">
+        <v>1</v>
+      </c>
+      <c r="L7" s="7">
+        <v>1</v>
+      </c>
+      <c r="M7" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="O6" s="6" t="s">
+      <c r="N7" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="O7" s="6" t="str">
+        <f>_xlfn.CONCAT("{",_xlfn.TEXTJOIN(",",TRUE,P7:R7),"}")</f>
+        <v>{{close_to_target,1000,combine,5,10,10},{default_rotate, 1000, combine, 180, 180},{dash,2000,combine,20,20,false,{fixed_timing,1,3,true}}}</v>
+      </c>
+      <c r="P7" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="P6" s="6" t="s">
+      <c r="Q7" s="6" t="s">
         <v>26</v>
+      </c>
+      <c r="R7" s="6" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="D1:P1"/>
-    <mergeCell ref="D2:P2"/>
+  <mergeCells count="3">
+    <mergeCell ref="D1:O1"/>
+    <mergeCell ref="D2:O2"/>
     <mergeCell ref="M3:N3"/>
-    <mergeCell ref="O3:P3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
feat: Enhance marble abilities configuration and initialization
- Added new ability configurations for MarbleSyncScale, MarbleSyncMass, MarbleDamagePipeline, MarbleHealPipeline, MarbleShieldHealPipeline, MarbleReceiveDamage, MarbleAddHeal, MarbleAddExp, MarbleDeath, MarbleLevelUp, MarbleGetTarget, MarbleMovement, and MarbleRotation.
- Updated marble.xml and marble_ability.xml to include new ability configurations.
- Refactored MarbleFactory to initialize abilities using the new configuration classes.
- Improved JSON configuration for marble abilities to include priority settings.
- Adjusted related classes to support the new configuration structure, enhancing maintainability and readability.
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/marble.xlsx
+++ b/Configs/GameConfig/Datas/marble.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="51">
   <si>
     <t>##var</t>
   </si>
@@ -51,6 +51,45 @@
   </si>
   <si>
     <t>level</t>
+  </si>
+  <si>
+    <t>sync_scale</t>
+  </si>
+  <si>
+    <t>sync_mass</t>
+  </si>
+  <si>
+    <t>damage_pipeline</t>
+  </si>
+  <si>
+    <t>heal_pipeline</t>
+  </si>
+  <si>
+    <t>shield_heal_pipeline</t>
+  </si>
+  <si>
+    <t>receive_damage</t>
+  </si>
+  <si>
+    <t>add_heal</t>
+  </si>
+  <si>
+    <t>add_exp</t>
+  </si>
+  <si>
+    <t>death</t>
+  </si>
+  <si>
+    <t>level_up</t>
+  </si>
+  <si>
+    <t>get_target</t>
+  </si>
+  <si>
+    <t>movement</t>
+  </si>
+  <si>
+    <t>rotation</t>
   </si>
   <si>
     <t>upgrade_exp</t>
@@ -1261,24 +1300,36 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:R9"/>
+  <dimension ref="A1:AF9"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="9" style="4"/>
     <col min="2" max="2" width="9" style="5"/>
     <col min="3" max="3" width="8.09090909090909" style="4" customWidth="1"/>
     <col min="4" max="4" width="22.1818181818182" style="4" customWidth="1"/>
-    <col min="5" max="5" width="12.9090909090909" style="6" customWidth="1"/>
-    <col min="6" max="11" width="9" style="6"/>
-    <col min="12" max="12" width="9" style="7"/>
-    <col min="13" max="14" width="18.5454545454545" style="6" customWidth="1"/>
-    <col min="15" max="15" width="168.636363636364" style="6" customWidth="1"/>
-    <col min="16" max="16" width="47.1818181818182" customWidth="1"/>
-    <col min="17" max="17" width="50.8181818181818" customWidth="1"/>
-    <col min="18" max="18" width="66.8181818181818" customWidth="1"/>
+    <col min="5" max="5" width="12.8181818181818" style="4" customWidth="1"/>
+    <col min="6" max="6" width="11.5454545454545" style="4" customWidth="1"/>
+    <col min="7" max="8" width="18.9090909090909" style="4" customWidth="1"/>
+    <col min="9" max="9" width="25.0909090909091" style="4" customWidth="1"/>
+    <col min="10" max="10" width="17.7272727272727" style="4" customWidth="1"/>
+    <col min="11" max="11" width="10.3636363636364" style="4" customWidth="1"/>
+    <col min="12" max="12" width="9.18181818181818" style="4" customWidth="1"/>
+    <col min="13" max="13" width="7" style="4" customWidth="1"/>
+    <col min="14" max="14" width="10.3636363636364" style="4" customWidth="1"/>
+    <col min="15" max="15" width="12.8181818181818" style="4" customWidth="1"/>
+    <col min="16" max="17" width="10.3636363636364" style="4" customWidth="1"/>
+    <col min="18" max="18" width="22.1818181818182" style="4" customWidth="1"/>
+    <col min="19" max="19" width="12.9090909090909" style="6" customWidth="1"/>
+    <col min="20" max="25" width="9" style="6"/>
+    <col min="26" max="26" width="9" style="7"/>
+    <col min="27" max="28" width="18.5454545454545" style="6" customWidth="1"/>
+    <col min="29" max="29" width="168.636363636364" style="6" customWidth="1"/>
+    <col min="30" max="30" width="47.1818181818182" customWidth="1"/>
+    <col min="31" max="31" width="50.8181818181818" customWidth="1"/>
+    <col min="32" max="32" width="66.8181818181818" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:18">
+    <row r="1" s="1" customFormat="1" spans="1:32">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -1299,13 +1350,27 @@
       <c r="J1" s="11"/>
       <c r="K1" s="11"/>
       <c r="L1" s="11"/>
-      <c r="M1" s="12"/>
-      <c r="N1" s="12"/>
-      <c r="O1" s="12"/>
-      <c r="P1" s="13"/>
-      <c r="Q1" s="13"/>
+      <c r="M1" s="11"/>
+      <c r="N1" s="11"/>
+      <c r="O1" s="11"/>
+      <c r="P1" s="11"/>
+      <c r="Q1" s="11"/>
+      <c r="R1" s="11"/>
+      <c r="S1" s="11"/>
+      <c r="T1" s="11"/>
+      <c r="U1" s="11"/>
+      <c r="V1" s="11"/>
+      <c r="W1" s="11"/>
+      <c r="X1" s="11"/>
+      <c r="Y1" s="11"/>
+      <c r="Z1" s="11"/>
+      <c r="AA1" s="12"/>
+      <c r="AB1" s="12"/>
+      <c r="AC1" s="12"/>
+      <c r="AD1" s="13"/>
+      <c r="AE1" s="13"/>
     </row>
-    <row r="2" s="2" customFormat="1" spans="1:18">
+    <row r="2" s="2" customFormat="1" spans="1:32">
       <c r="A2" s="14" t="s">
         <v>4</v>
       </c>
@@ -1325,12 +1390,26 @@
       <c r="I2" s="17"/>
       <c r="J2" s="17"/>
       <c r="K2" s="17"/>
-      <c r="L2" s="18"/>
-      <c r="M2" s="16"/>
-      <c r="N2" s="16"/>
-      <c r="O2" s="16"/>
+      <c r="L2" s="17"/>
+      <c r="M2" s="17"/>
+      <c r="N2" s="17"/>
+      <c r="O2" s="17"/>
+      <c r="P2" s="17"/>
+      <c r="Q2" s="17"/>
+      <c r="R2" s="17"/>
+      <c r="S2" s="17"/>
+      <c r="T2" s="17"/>
+      <c r="U2" s="17"/>
+      <c r="V2" s="17"/>
+      <c r="W2" s="17"/>
+      <c r="X2" s="17"/>
+      <c r="Y2" s="17"/>
+      <c r="Z2" s="18"/>
+      <c r="AA2" s="16"/>
+      <c r="AB2" s="16"/>
+      <c r="AC2" s="16"/>
     </row>
-    <row r="3" s="1" customFormat="1" spans="1:18">
+    <row r="3" s="1" customFormat="1" spans="1:32">
       <c r="A3" s="12" t="s">
         <v>0</v>
       </c>
@@ -1339,279 +1418,503 @@
       <c r="D3" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="21" t="s">
+      <c r="E3" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="21" t="s">
+      <c r="F3" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="G3" s="21" t="s">
+      <c r="G3" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="21" t="s">
+      <c r="H3" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="I3" s="21" t="s">
+      <c r="I3" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="J3" s="21" t="s">
+      <c r="J3" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="K3" s="21" t="s">
+      <c r="K3" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="L3" s="22" t="s">
+      <c r="L3" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="M3" s="23" t="s">
+      <c r="M3" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="N3" s="23"/>
-      <c r="O3" s="24" t="s">
+      <c r="N3" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="P3" s="25"/>
-      <c r="Q3" s="25"/>
+      <c r="O3" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="P3" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q3" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="R3" s="20"/>
+      <c r="S3" s="21" t="s">
+        <v>21</v>
+      </c>
+      <c r="T3" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="U3" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="V3" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="W3" s="21" t="s">
+        <v>25</v>
+      </c>
+      <c r="X3" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="Y3" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z3" s="22" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA3" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB3" s="23"/>
+      <c r="AC3" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="AD3" s="25"/>
+      <c r="AE3" s="25"/>
     </row>
-    <row r="4" s="1" customFormat="1" spans="1:18">
+    <row r="4" s="1" customFormat="1" spans="1:32">
       <c r="A4" s="12" t="s">
         <v>0</v>
       </c>
       <c r="B4" s="19"/>
       <c r="C4" s="20"/>
       <c r="D4" s="20"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="21"/>
-      <c r="G4" s="21"/>
-      <c r="H4" s="21"/>
-      <c r="I4" s="21"/>
-      <c r="J4" s="21"/>
-      <c r="K4" s="21"/>
-      <c r="L4" s="22"/>
-      <c r="M4" s="23"/>
-      <c r="N4" s="23"/>
-      <c r="O4" s="26"/>
-      <c r="P4" s="25"/>
-      <c r="Q4" s="25"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="20"/>
+      <c r="H4" s="20"/>
+      <c r="I4" s="20"/>
+      <c r="J4" s="20"/>
+      <c r="K4" s="20"/>
+      <c r="L4" s="20"/>
+      <c r="M4" s="20"/>
+      <c r="N4" s="20"/>
+      <c r="O4" s="20"/>
+      <c r="P4" s="20"/>
+      <c r="Q4" s="20"/>
+      <c r="R4" s="20"/>
+      <c r="S4" s="21"/>
+      <c r="T4" s="21"/>
+      <c r="U4" s="21"/>
+      <c r="V4" s="21"/>
+      <c r="W4" s="21"/>
+      <c r="X4" s="21"/>
+      <c r="Y4" s="21"/>
+      <c r="Z4" s="22"/>
+      <c r="AA4" s="23"/>
+      <c r="AB4" s="23"/>
+      <c r="AC4" s="26"/>
+      <c r="AD4" s="25"/>
+      <c r="AE4" s="25"/>
     </row>
-    <row r="5" s="3" customFormat="1" spans="1:18">
+    <row r="5" s="3" customFormat="1" spans="1:32">
       <c r="A5" s="27" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="B5" s="28"/>
       <c r="C5" s="29"/>
       <c r="D5" s="29"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="30"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="30"/>
-      <c r="J5" s="30"/>
-      <c r="K5" s="30"/>
-      <c r="L5" s="31"/>
-      <c r="M5" s="30"/>
-      <c r="N5" s="30"/>
-      <c r="O5" s="32" t="s">
-        <v>19</v>
+      <c r="E5" s="29"/>
+      <c r="F5" s="29"/>
+      <c r="G5" s="29"/>
+      <c r="H5" s="29"/>
+      <c r="I5" s="29"/>
+      <c r="J5" s="29"/>
+      <c r="K5" s="29"/>
+      <c r="L5" s="29"/>
+      <c r="M5" s="29"/>
+      <c r="N5" s="29"/>
+      <c r="O5" s="29"/>
+      <c r="P5" s="29"/>
+      <c r="Q5" s="29"/>
+      <c r="R5" s="29"/>
+      <c r="S5" s="30"/>
+      <c r="T5" s="30"/>
+      <c r="U5" s="30"/>
+      <c r="V5" s="30"/>
+      <c r="W5" s="30"/>
+      <c r="X5" s="30"/>
+      <c r="Y5" s="30"/>
+      <c r="Z5" s="31"/>
+      <c r="AA5" s="30"/>
+      <c r="AB5" s="30"/>
+      <c r="AC5" s="32" t="s">
+        <v>32</v>
       </c>
     </row>
-    <row r="6" customHeight="1" spans="1:18">
+    <row r="6" customHeight="1" spans="1:32">
       <c r="B6" s="5" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="E6" s="6">
+        <v>35</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="L6" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="M6" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="N6" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="O6" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="P6" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q6" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="S6" s="6">
         <v>100</v>
       </c>
-      <c r="F6" s="6">
+      <c r="T6" s="6">
         <v>100</v>
       </c>
-      <c r="G6" s="6">
+      <c r="U6" s="6">
         <v>100</v>
       </c>
-      <c r="H6" s="6">
+      <c r="V6" s="6">
         <v>10</v>
       </c>
-      <c r="I6" s="6">
+      <c r="W6" s="6">
         <v>5</v>
       </c>
-      <c r="J6" s="6">
+      <c r="X6" s="6">
         <v>8</v>
       </c>
-      <c r="K6" s="6">
+      <c r="Y6" s="6">
         <v>1</v>
       </c>
-      <c r="L6" s="7">
+      <c r="Z6" s="7">
         <v>1</v>
       </c>
-      <c r="M6" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="N6" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="O6" s="6" t="str">
-        <f>_xlfn.CONCAT("{",_xlfn.TEXTJOIN(",",TRUE,P6:R6),"}")</f>
+      <c r="AA6" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="AB6" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="AC6" s="6" t="str">
+        <f>_xlfn.CONCAT("{",_xlfn.TEXTJOIN(",",TRUE,AD6:AF6),"}")</f>
         <v>{{close_to_target,1000,combine,5,10,10},{default_rotate, 1000, combine, 180, 180},{dash,2000,combine,20,20,false,{random_range_timing,1,1,1,3,true}}}</v>
       </c>
-      <c r="P6" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q6" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="R6" s="6" t="s">
-        <v>27</v>
+      <c r="AD6" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE6" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="AF6" s="6" t="s">
+        <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:18">
+    <row r="7" spans="1:32">
       <c r="D7" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="E7" s="6">
+        <v>41</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="K7" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="L7" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="M7" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="N7" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="O7" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="P7" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q7" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="S7" s="6">
         <v>150</v>
       </c>
-      <c r="F7" s="6">
+      <c r="T7" s="6">
         <v>150</v>
       </c>
-      <c r="G7" s="6">
+      <c r="U7" s="6">
         <v>150</v>
       </c>
-      <c r="H7" s="6">
+      <c r="V7" s="6">
         <v>10</v>
       </c>
-      <c r="I7" s="6">
+      <c r="W7" s="6">
         <v>5</v>
       </c>
-      <c r="J7" s="6">
+      <c r="X7" s="6">
         <v>8</v>
       </c>
-      <c r="K7" s="6">
+      <c r="Y7" s="6">
         <v>1</v>
       </c>
-      <c r="L7" s="7">
+      <c r="Z7" s="7">
         <v>1</v>
       </c>
-      <c r="M7" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N7" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="O7" s="6" t="str">
-        <f>_xlfn.CONCAT("{",_xlfn.TEXTJOIN(",",TRUE,P7:R7),"}")</f>
+      <c r="AA7" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="AB7" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="AC7" s="6" t="str">
+        <f>_xlfn.CONCAT("{",_xlfn.TEXTJOIN(",",TRUE,AD7:AF7),"}")</f>
         <v>{{close_to_target,1000,combine,5,10,10},{default_rotate, 1000, combine, 180, 180},{dash,2000,combine,20,20,false,{random_range_timing,1,1,1,3,true}}}</v>
       </c>
-      <c r="P7" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q7" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="R7" s="6" t="s">
-        <v>27</v>
+      <c r="AD7" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE7" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="AF7" s="6" t="s">
+        <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:18">
+    <row r="8" spans="1:32">
       <c r="B8" s="5" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="E8" s="6">
+        <v>35</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="L8" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="M8" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="N8" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="O8" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="P8" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q8" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="S8" s="6">
         <v>100</v>
       </c>
-      <c r="F8" s="6">
+      <c r="T8" s="6">
         <v>100</v>
       </c>
-      <c r="G8" s="6">
+      <c r="U8" s="6">
         <v>100</v>
       </c>
-      <c r="H8" s="6">
+      <c r="V8" s="6">
         <v>10</v>
       </c>
-      <c r="I8" s="6">
+      <c r="W8" s="6">
         <v>5</v>
       </c>
-      <c r="J8" s="6">
+      <c r="X8" s="6">
         <v>8</v>
       </c>
-      <c r="K8" s="6">
+      <c r="Y8" s="6">
         <v>1</v>
       </c>
-      <c r="L8" s="7">
+      <c r="Z8" s="7">
         <v>1</v>
       </c>
-      <c r="M8" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="O8" s="6" t="str">
-        <f>_xlfn.CONCAT("{",_xlfn.TEXTJOIN(",",TRUE,P8:R8),"}")</f>
+      <c r="AA8" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="AC8" s="6" t="str">
+        <f>_xlfn.CONCAT("{",_xlfn.TEXTJOIN(",",TRUE,AD8:AF8),"}")</f>
         <v>{{close_to_target,1000,combine,8,10,10},{face_target_direction, 1000, combine, {1,0}, 20, 20, {fixed_timing, 10000, 1, true}}}</v>
       </c>
-      <c r="P8" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="Q8" s="6" t="s">
-        <v>35</v>
+      <c r="AD8" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="AE8" s="6" t="s">
+        <v>48</v>
       </c>
     </row>
-    <row r="9" spans="1:18">
+    <row r="9" spans="1:32">
       <c r="D9" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="E9" s="6">
+        <v>41</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="L9" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="M9" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="N9" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="O9" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="P9" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q9" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="S9" s="6">
         <v>150</v>
       </c>
-      <c r="F9" s="6">
+      <c r="T9" s="6">
         <v>150</v>
       </c>
-      <c r="G9" s="6">
+      <c r="U9" s="6">
         <v>150</v>
       </c>
-      <c r="H9" s="6">
+      <c r="V9" s="6">
         <v>10</v>
       </c>
-      <c r="I9" s="6">
+      <c r="W9" s="6">
         <v>5</v>
       </c>
-      <c r="J9" s="6">
+      <c r="X9" s="6">
         <v>8</v>
       </c>
-      <c r="K9" s="6">
+      <c r="Y9" s="6">
         <v>1</v>
       </c>
-      <c r="L9" s="7">
+      <c r="Z9" s="7">
         <v>1</v>
       </c>
-      <c r="M9" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="O9" s="6" t="str">
-        <f>_xlfn.CONCAT("{",_xlfn.TEXTJOIN(",",TRUE,P9:R9),"}")</f>
+      <c r="AA9" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="AC9" s="6" t="str">
+        <f>_xlfn.CONCAT("{",_xlfn.TEXTJOIN(",",TRUE,AD9:AF9),"}")</f>
         <v>{{close_to_target,1000,combine,8,10,10},{face_target_direction, 1000, combine, {1,0}, 60, 60, {fixed_timing, 10000, 1, true}}}</v>
       </c>
-      <c r="P9" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="Q9" s="6" t="s">
-        <v>37</v>
+      <c r="AD9" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="AE9" s="6" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="D1:O1"/>
-    <mergeCell ref="D2:O2"/>
-    <mergeCell ref="M3:N3"/>
+    <mergeCell ref="D1:AC1"/>
+    <mergeCell ref="D2:AC2"/>
+    <mergeCell ref="AA3:AB3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
feat: Implement projectile knockback ability and enhance combat interactions
- Added a new ProjectileKnockbackAbility to apply knockback effects upon projectile hits.
- Introduced ProjectileHitContext for managing hit interactions and improved damage handling in ProjectileDamageAbility.
- Updated configuration files to support knockback settings and integrated new ability into the projectile factory.
- Refactored existing projectile abilities to utilize the new hit context for better maintainability and clarity in combat logic.
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/marble.xlsx
+++ b/Configs/GameConfig/Datas/marble.xlsx
@@ -1621,7 +1621,7 @@
         <v>100</v>
       </c>
       <c r="V6" s="6">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="W6" s="6">
         <v>5</v>
@@ -1708,7 +1708,7 @@
         <v>150</v>
       </c>
       <c r="V7" s="6">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="W7" s="6">
         <v>5</v>
@@ -1801,7 +1801,7 @@
         <v>100</v>
       </c>
       <c r="V8" s="6">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="W8" s="6">
         <v>5</v>
@@ -1882,7 +1882,7 @@
         <v>150</v>
       </c>
       <c r="V9" s="6">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="W9" s="6">
         <v>5</v>

</xml_diff>

<commit_message>
feat: Update equipment configurations and refine combat mechanics
- Updated equip.xlsx and marble.xlsx files to reflect new equipment data.
- Adjusted shield and sword prefab settings for improved combat dynamics, including motor force and angle limits.
- Enhanced EquipmentFactory to support parent transform assignment during equipment creation.
- Modified gameplay_combat_tbmarble.json to improve marble combat configurations.
- Refactored EquipmentBrokenAbility to apply drag settings to all child rigidbodies.
- Updated EquipmentMountAbility to refine equipment attachment logic and transform handling.
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/marble.xlsx
+++ b/Configs/GameConfig/Datas/marble.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="55">
   <si>
     <t>##var</t>
   </si>
@@ -189,6 +189,9 @@
   </si>
   <si>
     <t>spear,0,bottom</t>
+  </si>
+  <si>
+    <t>{face_target_direction, 1000, combine, {1,0}, 360, 180, {fixed_timing, 10000, 1, true}}</t>
   </si>
 </sst>
 </file>
@@ -581,7 +584,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -645,6 +648,17 @@
       </left>
       <right/>
       <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
@@ -774,7 +788,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -786,34 +800,34 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -898,7 +912,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -968,14 +982,20 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1309,7 +1329,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AF10"/>
+  <dimension ref="A1:AG10"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="9" style="4"/>
@@ -1331,14 +1351,14 @@
     <col min="19" max="19" width="12.9090909090909" style="6" customWidth="1"/>
     <col min="20" max="25" width="9" style="6"/>
     <col min="26" max="26" width="9" style="7"/>
-    <col min="27" max="28" width="18.5454545454545" style="6" customWidth="1"/>
-    <col min="29" max="29" width="168.636363636364" style="6" customWidth="1"/>
-    <col min="30" max="30" width="88.9090909090909" customWidth="1"/>
-    <col min="31" max="31" width="50.8181818181818" customWidth="1"/>
-    <col min="32" max="32" width="66.8181818181818" customWidth="1"/>
+    <col min="27" max="29" width="18.5454545454545" style="6" customWidth="1"/>
+    <col min="30" max="30" width="168.636363636364" style="6" customWidth="1"/>
+    <col min="31" max="31" width="88.9090909090909" customWidth="1"/>
+    <col min="32" max="32" width="50.8181818181818" customWidth="1"/>
+    <col min="33" max="33" width="66.8181818181818" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:32">
+    <row r="1" s="1" customFormat="1" spans="1:33">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -1376,10 +1396,11 @@
       <c r="AA1" s="12"/>
       <c r="AB1" s="12"/>
       <c r="AC1" s="12"/>
-      <c r="AD1" s="13"/>
+      <c r="AD1" s="12"/>
       <c r="AE1" s="13"/>
+      <c r="AF1" s="13"/>
     </row>
-    <row r="2" s="2" customFormat="1" spans="1:32">
+    <row r="2" s="2" customFormat="1" spans="1:33">
       <c r="A2" s="14" t="s">
         <v>4</v>
       </c>
@@ -1417,8 +1438,9 @@
       <c r="AA2" s="16"/>
       <c r="AB2" s="16"/>
       <c r="AC2" s="16"/>
+      <c r="AD2" s="16"/>
     </row>
-    <row r="3" s="1" customFormat="1" spans="1:32">
+    <row r="3" s="1" customFormat="1" spans="1:33">
       <c r="A3" s="12" t="s">
         <v>0</v>
       </c>
@@ -1494,14 +1516,15 @@
       <c r="AA3" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="AB3" s="23"/>
-      <c r="AC3" s="24" t="s">
+      <c r="AB3" s="24"/>
+      <c r="AC3" s="24"/>
+      <c r="AD3" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="AD3" s="25"/>
-      <c r="AE3" s="25"/>
+      <c r="AE3" s="26"/>
+      <c r="AF3" s="26"/>
     </row>
-    <row r="4" s="1" customFormat="1" spans="1:32">
+    <row r="4" s="1" customFormat="1" spans="1:33">
       <c r="A4" s="12" t="s">
         <v>0</v>
       </c>
@@ -1530,48 +1553,50 @@
       <c r="X4" s="21"/>
       <c r="Y4" s="21"/>
       <c r="Z4" s="22"/>
-      <c r="AA4" s="23"/>
-      <c r="AB4" s="23"/>
-      <c r="AC4" s="26"/>
-      <c r="AD4" s="25"/>
-      <c r="AE4" s="25"/>
+      <c r="AA4" s="27"/>
+      <c r="AB4" s="27"/>
+      <c r="AC4" s="27"/>
+      <c r="AD4" s="28"/>
+      <c r="AE4" s="26"/>
+      <c r="AF4" s="26"/>
     </row>
-    <row r="5" s="3" customFormat="1" spans="1:32">
-      <c r="A5" s="27" t="s">
+    <row r="5" s="3" customFormat="1" spans="1:33">
+      <c r="A5" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="B5" s="28"/>
-      <c r="C5" s="29"/>
-      <c r="D5" s="29"/>
-      <c r="E5" s="29"/>
-      <c r="F5" s="29"/>
-      <c r="G5" s="29"/>
-      <c r="H5" s="29"/>
-      <c r="I5" s="29"/>
-      <c r="J5" s="29"/>
-      <c r="K5" s="29"/>
-      <c r="L5" s="29"/>
-      <c r="M5" s="29"/>
-      <c r="N5" s="29"/>
-      <c r="O5" s="29"/>
-      <c r="P5" s="29"/>
-      <c r="Q5" s="29"/>
-      <c r="R5" s="29"/>
-      <c r="S5" s="30"/>
-      <c r="T5" s="30"/>
-      <c r="U5" s="30"/>
-      <c r="V5" s="30"/>
-      <c r="W5" s="30"/>
-      <c r="X5" s="30"/>
-      <c r="Y5" s="30"/>
-      <c r="Z5" s="31"/>
-      <c r="AA5" s="30"/>
-      <c r="AB5" s="30"/>
-      <c r="AC5" s="32" t="s">
+      <c r="B5" s="30"/>
+      <c r="C5" s="31"/>
+      <c r="D5" s="31"/>
+      <c r="E5" s="31"/>
+      <c r="F5" s="31"/>
+      <c r="G5" s="31"/>
+      <c r="H5" s="31"/>
+      <c r="I5" s="31"/>
+      <c r="J5" s="31"/>
+      <c r="K5" s="31"/>
+      <c r="L5" s="31"/>
+      <c r="M5" s="31"/>
+      <c r="N5" s="31"/>
+      <c r="O5" s="31"/>
+      <c r="P5" s="31"/>
+      <c r="Q5" s="31"/>
+      <c r="R5" s="31"/>
+      <c r="S5" s="32"/>
+      <c r="T5" s="32"/>
+      <c r="U5" s="32"/>
+      <c r="V5" s="32"/>
+      <c r="W5" s="32"/>
+      <c r="X5" s="32"/>
+      <c r="Y5" s="32"/>
+      <c r="Z5" s="33"/>
+      <c r="AA5" s="32"/>
+      <c r="AB5" s="32"/>
+      <c r="AC5" s="32"/>
+      <c r="AD5" s="34" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="6" customHeight="1" spans="1:32">
+    <row r="6" customHeight="1" spans="1:33">
       <c r="B6" s="5" t="s">
         <v>33</v>
       </c>
@@ -1650,21 +1675,21 @@
       <c r="AB6" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="AC6" s="6" t="str">
-        <f>_xlfn.CONCAT("{",_xlfn.TEXTJOIN(",",TRUE,AD6:AF6),"}")</f>
+      <c r="AD6" s="6" t="str">
+        <f>_xlfn.CONCAT("{",_xlfn.TEXTJOIN(",",TRUE,AE6:AG6),"}")</f>
         <v>{{close_to_target,1000,combine,5,10,10,{fixed_timing,5,5,true}},{default_rotate, 1000, combine, 180, 180},{dash,2000,combine,20,20,false,{random_range_timing,1,1,1,3,true}}}</v>
       </c>
-      <c r="AD6" s="6" t="s">
+      <c r="AE6" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="AE6" s="6" t="s">
+      <c r="AF6" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="AF6" s="6" t="s">
+      <c r="AG6" s="6" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:32">
+    <row r="7" spans="1:33">
       <c r="D7" s="4" t="s">
         <v>41</v>
       </c>
@@ -1737,21 +1762,21 @@
       <c r="AB7" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="AC7" s="6" t="str">
-        <f>_xlfn.CONCAT("{",_xlfn.TEXTJOIN(",",TRUE,AD7:AF7),"}")</f>
+      <c r="AD7" s="6" t="str">
+        <f>_xlfn.CONCAT("{",_xlfn.TEXTJOIN(",",TRUE,AE7:AG7),"}")</f>
         <v>{{close_to_target,1000,combine,5,10,10,{fixed_timing,5,5,true}},{default_rotate, 1000, combine, 180, 180},{dash,2000,combine,20,20,false,{random_range_timing,1,1,1,3,true}}}</v>
       </c>
-      <c r="AD7" s="6" t="s">
+      <c r="AE7" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="AE7" s="6" t="s">
+      <c r="AF7" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="AF7" s="6" t="s">
+      <c r="AG7" s="6" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:32">
+    <row r="8" spans="1:33">
       <c r="B8" s="5" t="s">
         <v>44</v>
       </c>
@@ -1827,18 +1852,18 @@
       <c r="AA8" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="AC8" s="6" t="str">
-        <f>_xlfn.CONCAT("{",_xlfn.TEXTJOIN(",",TRUE,AD8:AF8),"}")</f>
+      <c r="AD8" s="6" t="str">
+        <f>_xlfn.CONCAT("{",_xlfn.TEXTJOIN(",",TRUE,AE8:AG8),"}")</f>
         <v>{{keep_away_from_target,1000,combine,5,10,10,{fixed_timing,5,3,true}},{face_target_direction, 1000, combine, {1,0}, 20, 20, {fixed_timing, 10000, 1, true}}}</v>
       </c>
-      <c r="AD8" s="6" t="s">
+      <c r="AE8" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="AE8" s="6" t="s">
+      <c r="AF8" s="6" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="9" spans="1:32">
+    <row r="9" spans="1:33">
       <c r="D9" s="4" t="s">
         <v>41</v>
       </c>
@@ -1908,18 +1933,18 @@
       <c r="AA9" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="AC9" s="6" t="str">
-        <f>_xlfn.CONCAT("{",_xlfn.TEXTJOIN(",",TRUE,AD9:AF9),"}")</f>
+      <c r="AD9" s="6" t="str">
+        <f>_xlfn.CONCAT("{",_xlfn.TEXTJOIN(",",TRUE,AE9:AG9),"}")</f>
         <v>{{keep_away_from_target,1000,combine,5,10,10,{fixed_timing,5,3,true}},{face_target_direction, 1000, combine, {1,0}, 60, 60, {fixed_timing, 10000, 1, true}}}</v>
       </c>
-      <c r="AD9" s="6" t="s">
+      <c r="AE9" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="AE9" s="6" t="s">
+      <c r="AF9" s="6" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:32">
+    <row r="10" spans="1:33">
       <c r="B10" s="5" t="s">
         <v>51</v>
       </c>
@@ -1996,25 +2021,26 @@
         <v>53</v>
       </c>
       <c r="AB10" s="6"/>
-      <c r="AC10" s="6" t="str">
-        <f>_xlfn.CONCAT("{",_xlfn.TEXTJOIN(",",TRUE,AD10:AF10),"}")</f>
-        <v>{{close_to_target,1000,combine,5,10,10,{fixed_timing,5,5,true}},{face_target_direction, 1000, combine, {1,0}, 20, 20, {fixed_timing, 10000, 1, true}},{dash,2000,combine,20,20,false,{random_range_timing,1,1,1,3,true}}}</v>
-      </c>
-      <c r="AD10" s="6" t="s">
+      <c r="AC10" s="6"/>
+      <c r="AD10" s="6" t="str">
+        <f>_xlfn.CONCAT("{",_xlfn.TEXTJOIN(",",TRUE,AE10:AG10),"}")</f>
+        <v>{{close_to_target,1000,combine,5,10,10,{fixed_timing,5,5,true}},{face_target_direction, 1000, combine, {1,0}, 360, 180, {fixed_timing, 10000, 1, true}},{dash,2000,combine,20,20,false,{random_range_timing,1,1,1,3,true}}}</v>
+      </c>
+      <c r="AE10" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="AE10" s="6" t="s">
-        <v>48</v>
-      </c>
       <c r="AF10" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="AG10" s="6" t="s">
         <v>40</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="D1:AC1"/>
-    <mergeCell ref="D2:AC2"/>
-    <mergeCell ref="AA3:AB3"/>
+    <mergeCell ref="D1:AD1"/>
+    <mergeCell ref="D2:AD2"/>
+    <mergeCell ref="AA3:AC3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
feat: Update equipment prefabs and add sorting groups
- Modified bow, shield, spear, sword, and marble prefabs to include new sorting group components for improved rendering order.
- Updated marble.xlsx to reflect changes in equipment configurations.
- Enhanced arrow prefab with a new sorting group component for better visual management.
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/marble.xlsx
+++ b/Configs/GameConfig/Datas/marble.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="56">
   <si>
     <t>##var</t>
   </si>
@@ -123,6 +123,9 @@
   </si>
   <si>
     <t>##</t>
+  </si>
+  <si>
+    <t>装备id,等级，装备位置</t>
   </si>
   <si>
     <t>type,priority</t>
@@ -1589,61 +1592,63 @@
       <c r="X5" s="32"/>
       <c r="Y5" s="32"/>
       <c r="Z5" s="33"/>
-      <c r="AA5" s="32"/>
+      <c r="AA5" s="32" t="s">
+        <v>32</v>
+      </c>
       <c r="AB5" s="32"/>
       <c r="AC5" s="32"/>
       <c r="AD5" s="34" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" customHeight="1" spans="1:33">
       <c r="B6" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="M6" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="N6" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="O6" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P6" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q6" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="S6" s="6">
         <v>100</v>
@@ -1670,67 +1675,67 @@
         <v>1</v>
       </c>
       <c r="AA6" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="AB6" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="AD6" s="6" t="str">
         <f>_xlfn.CONCAT("{",_xlfn.TEXTJOIN(",",TRUE,AE6:AG6),"}")</f>
         <v>{{close_to_target,1000,combine,5,10,10,{fixed_timing,5,5,true}},{default_rotate, 1000, combine, 180, 180},{dash,2000,combine,20,20,false,{random_range_timing,1,1,1,3,true}}}</v>
       </c>
       <c r="AE6" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="AF6" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="AG6" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:33">
       <c r="D7" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="K7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="L7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="M7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="N7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="O7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q7" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="S7" s="6">
         <v>150</v>
@@ -1757,73 +1762,73 @@
         <v>1</v>
       </c>
       <c r="AA7" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="AB7" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="AD7" s="6" t="str">
         <f>_xlfn.CONCAT("{",_xlfn.TEXTJOIN(",",TRUE,AE7:AG7),"}")</f>
         <v>{{close_to_target,1000,combine,5,10,10,{fixed_timing,5,5,true}},{default_rotate, 1000, combine, 180, 180},{dash,2000,combine,20,20,false,{random_range_timing,1,1,1,3,true}}}</v>
       </c>
       <c r="AE7" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="AF7" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="AG7" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" spans="1:33">
       <c r="B8" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="K8" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="L8" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="M8" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="N8" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="O8" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P8" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q8" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="S8" s="6">
         <v>100</v>
@@ -1850,61 +1855,61 @@
         <v>1</v>
       </c>
       <c r="AA8" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="AD8" s="6" t="str">
         <f>_xlfn.CONCAT("{",_xlfn.TEXTJOIN(",",TRUE,AE8:AG8),"}")</f>
         <v>{{keep_away_from_target,1000,combine,5,10,10,{fixed_timing,5,3,true}},{face_target_direction, 1000, combine, {1,0}, 20, 20, {fixed_timing, 10000, 1, true}}}</v>
       </c>
       <c r="AE8" s="6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="AF8" s="6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:33">
       <c r="D9" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="K9" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="L9" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="M9" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="N9" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="O9" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P9" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q9" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="S9" s="6">
         <v>150</v>
@@ -1931,67 +1936,67 @@
         <v>1</v>
       </c>
       <c r="AA9" s="6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AD9" s="6" t="str">
         <f>_xlfn.CONCAT("{",_xlfn.TEXTJOIN(",",TRUE,AE9:AG9),"}")</f>
         <v>{{keep_away_from_target,1000,combine,5,10,10,{fixed_timing,5,3,true}},{face_target_direction, 1000, combine, {1,0}, 60, 60, {fixed_timing, 10000, 1, true}}}</v>
       </c>
       <c r="AE9" s="6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="AF9" s="6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="10" spans="1:33">
       <c r="B10" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="L10" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="M10" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="N10" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="O10" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="P10" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="Q10" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="S10" s="6">
         <v>100</v>
@@ -2018,7 +2023,7 @@
         <v>1</v>
       </c>
       <c r="AA10" s="6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="AB10" s="6"/>
       <c r="AC10" s="6"/>
@@ -2027,13 +2032,13 @@
         <v>{{close_to_target,1000,combine,5,10,10,{fixed_timing,5,5,true}},{face_target_direction, 1000, combine, {1,0}, 360, 180, {fixed_timing, 10000, 1, true}},{dash,2000,combine,20,20,false,{random_range_timing,1,1,1,3,true}}}</v>
       </c>
       <c r="AE10" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="AF10" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="AG10" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: Correct marble configuration and enhance UI layout
- Fixed the config_id for "soldier" in gameplay_combat_tbmarble.json.
- Updated marble.xlsx to ensure consistency in equipment configurations.
- Adjusted UI layout in ExpeditionMainUI and Test.unity for improved visual presentation.
- Enhanced font asset settings to support new glyph metrics and improve text rendering.
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/marble.xlsx
+++ b/Configs/GameConfig/Datas/marble.xlsx
@@ -131,7 +131,7 @@
     <t>type,priority</t>
   </si>
   <si>
-    <t>solider</t>
+    <t>soldier</t>
   </si>
   <si>
     <t>士兵</t>
@@ -915,7 +915,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -989,9 +989,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1521,11 +1518,11 @@
       </c>
       <c r="AB3" s="24"/>
       <c r="AC3" s="24"/>
-      <c r="AD3" s="25" t="s">
+      <c r="AD3" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="AE3" s="26"/>
-      <c r="AF3" s="26"/>
+      <c r="AE3" s="25"/>
+      <c r="AF3" s="25"/>
     </row>
     <row r="4" s="1" customFormat="1" spans="1:33">
       <c r="A4" s="12" t="s">
@@ -1556,48 +1553,48 @@
       <c r="X4" s="21"/>
       <c r="Y4" s="21"/>
       <c r="Z4" s="22"/>
-      <c r="AA4" s="27"/>
-      <c r="AB4" s="27"/>
-      <c r="AC4" s="27"/>
-      <c r="AD4" s="28"/>
-      <c r="AE4" s="26"/>
-      <c r="AF4" s="26"/>
+      <c r="AA4" s="26"/>
+      <c r="AB4" s="26"/>
+      <c r="AC4" s="26"/>
+      <c r="AD4" s="27"/>
+      <c r="AE4" s="25"/>
+      <c r="AF4" s="25"/>
     </row>
     <row r="5" s="3" customFormat="1" spans="1:33">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="B5" s="30"/>
-      <c r="C5" s="31"/>
-      <c r="D5" s="31"/>
-      <c r="E5" s="31"/>
-      <c r="F5" s="31"/>
-      <c r="G5" s="31"/>
-      <c r="H5" s="31"/>
-      <c r="I5" s="31"/>
-      <c r="J5" s="31"/>
-      <c r="K5" s="31"/>
-      <c r="L5" s="31"/>
-      <c r="M5" s="31"/>
-      <c r="N5" s="31"/>
-      <c r="O5" s="31"/>
-      <c r="P5" s="31"/>
-      <c r="Q5" s="31"/>
-      <c r="R5" s="31"/>
-      <c r="S5" s="32"/>
-      <c r="T5" s="32"/>
-      <c r="U5" s="32"/>
-      <c r="V5" s="32"/>
-      <c r="W5" s="32"/>
-      <c r="X5" s="32"/>
-      <c r="Y5" s="32"/>
-      <c r="Z5" s="33"/>
-      <c r="AA5" s="32" t="s">
+      <c r="B5" s="29"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+      <c r="J5" s="30"/>
+      <c r="K5" s="30"/>
+      <c r="L5" s="30"/>
+      <c r="M5" s="30"/>
+      <c r="N5" s="30"/>
+      <c r="O5" s="30"/>
+      <c r="P5" s="30"/>
+      <c r="Q5" s="30"/>
+      <c r="R5" s="30"/>
+      <c r="S5" s="31"/>
+      <c r="T5" s="31"/>
+      <c r="U5" s="31"/>
+      <c r="V5" s="31"/>
+      <c r="W5" s="31"/>
+      <c r="X5" s="31"/>
+      <c r="Y5" s="31"/>
+      <c r="Z5" s="32"/>
+      <c r="AA5" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="AB5" s="32"/>
-      <c r="AC5" s="32"/>
-      <c r="AD5" s="34" t="s">
+      <c r="AB5" s="31"/>
+      <c r="AC5" s="31"/>
+      <c r="AD5" s="33" t="s">
         <v>33</v>
       </c>
     </row>
@@ -2025,8 +2022,6 @@
       <c r="AA10" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="AB10" s="6"/>
-      <c r="AC10" s="6"/>
       <c r="AD10" s="6" t="str">
         <f>_xlfn.CONCAT("{",_xlfn.TEXTJOIN(",",TRUE,AE10:AG10),"}")</f>
         <v>{{close_to_target,1000,combine,5,10,10,{fixed_timing,5,5,true}},{face_target_direction, 1000, combine, {1,0}, 360, 180, {fixed_timing, 10000, 1, true}},{dash,2000,combine,20,20,false,{random_range_timing,1,1,1,3,true}}}</v>

</xml_diff>